<commit_message>
docs: add test execution guide to root README.md
</commit_message>
<xml_diff>
--- a/test_and_result/output.xlsx
+++ b/test_and_result/output.xlsx
@@ -1681,22 +1681,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://mirka-online.com/9a-570-320-mirka-abranet-2-3-4-in-x-10yd-mesh-grip-roll-320g-qty-1.html</t>
+          <t>https://www.nainc.org/product/mirka-abranet-2-3-4-in-x-10-yd-320g-mesh-grip-roll/</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://mirka-online.com/9a-570-320-mirka-abranet-2-3-4-in-x-10yd-mesh-grip-roll-320g-qty-1.html</t>
+          <t>https://www.nainc.org/product/mirka-abranet-2-3-4-in-x-10-yd-320g-mesh-grip-roll/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://buymirka.com/products/mirka-abranet-2-75-grip-sanding-rolls-9a-570-series</t>
+          <t>https://www.zoro.com/mirka-mesh-grip-roll-275x30ft-p320-grit-9a-570-320/i/G1693227/</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://mirka-online.com/9a-570-320-mirka-abranet-2-3-4-in-x-10yd-mesh-grip-roll-320g-qty-1.html/documents/9A-570-320_manual.pdf</t>
+          <t>https://www.nainc.org/product/mirka-abranet-2-3-4-in-x-10-yd-320g-mesh-grip-roll//documents/9A-570-320_manual.pdf</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
@@ -1798,17 +1798,17 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>Mirka®, 9A-570-320, Sanding Disc</t>
+          <t>Mirka®, 9A-570-320, Sanding Disc, Aluminum</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>Mirka® Sanding Disc, 9 A, 2-3/4 in W x 30 in D, Additional Information: Abrasive Material: Aluminum Oxide Mesh, Backing Material: Polyamide Fabric Mesh, Material Application: Dust-Free Woodworking, Automotive, Composites, Disc Type: Grip Mesh Roll / Strip.</t>
+          <t>Mirka® Sanding Disc, 9 A, 2-3/4 in W x 30 in D, Aluminum, Additional Information: Abrasive Material: Aluminum Oxide Mesh, Backing Material: Polyamide Fabric Mesh, Material Application: Dust-Free Woodworking, Automotive, Composites, Disc Type: Grip Mesh Roll / Strip.</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>Sanding Disc</t>
+          <t>Sanding Disc, Aluminum</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
@@ -1828,92 +1828,92 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
+          <t>Material / Construction: Aluminum</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
           <t>Abrasive Material: Aluminum Oxide Mesh</t>
         </is>
       </c>
-      <c r="AG2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
         <is>
           <t>Backing Material: Polyamide Fabric Mesh</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr">
+      <c r="AI2" t="inlineStr">
         <is>
           <t>Material Application: Dust-Free Woodworking, Automotive, Composites</t>
         </is>
       </c>
-      <c r="AI2" t="inlineStr">
+      <c r="AJ2" t="inlineStr">
         <is>
           <t>Disc Type: Grip Mesh Roll / Strip</t>
         </is>
       </c>
-      <c r="AJ2" t="inlineStr">
+      <c r="AK2" t="inlineStr">
         <is>
           <t>Trade Name: Abranet®</t>
         </is>
       </c>
-      <c r="AK2" t="inlineStr">
+      <c r="AL2" t="inlineStr">
         <is>
           <t>Amperage Rating: 9 A</t>
         </is>
       </c>
-      <c r="AL2" t="inlineStr">
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>Grit: P320</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
         <is>
           <t>LENGTH: 2-3/4 in</t>
         </is>
       </c>
-      <c r="AM2" t="inlineStr">
+      <c r="AO2" t="inlineStr">
         <is>
           <t>WIDTH: 30 in</t>
         </is>
       </c>
-      <c r="AN2" t="inlineStr">
+      <c r="AP2" t="inlineStr">
         <is>
           <t>Warranty: 1 Year Manufacturer, 1 Year Labor and Parts</t>
         </is>
       </c>
-      <c r="AO2" t="inlineStr">
+      <c r="AQ2" t="inlineStr">
         <is>
           <t>Premium abrasive grain formulation for fast cutting action</t>
         </is>
       </c>
-      <c r="AP2" t="inlineStr">
+      <c r="AR2" t="inlineStr">
         <is>
           <t>Heavy-duty backing for superior tear resistance and extended lifespan</t>
         </is>
       </c>
-      <c r="AQ2" t="inlineStr">
+      <c r="AS2" t="inlineStr">
         <is>
           <t>Optimized for industrial metalworking, woodworking, and surface prep</t>
         </is>
       </c>
-      <c r="AR2" t="inlineStr">
+      <c r="AT2" t="inlineStr">
         <is>
           <t>Brand / Manufacturer: Mirka</t>
         </is>
       </c>
-      <c r="AS2" t="inlineStr">
+      <c r="AU2" t="inlineStr">
         <is>
           <t>Product Category: Sanding Disc</t>
         </is>
       </c>
-      <c r="AT2" t="inlineStr">
+      <c r="AV2" t="inlineStr">
         <is>
           <t>Primary Application: Commercial &amp; Residential Sanding Disc Applications</t>
         </is>
       </c>
-      <c r="AU2" t="inlineStr">
+      <c r="AW2" t="inlineStr">
         <is>
           <t>Standard Packaging: 1 Each</t>
-        </is>
-      </c>
-      <c r="AV2" t="inlineStr">
-        <is>
-          <t>Warranty Protection: 1 Year Manufacturer, 1 Year Labor and Parts</t>
-        </is>
-      </c>
-      <c r="AW2" t="inlineStr">
-        <is>
-          <t>Engineered for heavy-duty industrial performance and durability</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr"/>
@@ -1988,480 +1988,488 @@
       <c r="BO2" t="inlineStr"/>
       <c r="BP2" t="inlineStr">
         <is>
-          <t>Selling Qty</t>
+          <t>Grit</t>
         </is>
       </c>
       <c r="BQ2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>P320</t>
         </is>
       </c>
       <c r="BR2" t="inlineStr"/>
       <c r="BS2" t="inlineStr">
         <is>
-          <t>Standard Packaging Information</t>
+          <t>Material</t>
         </is>
       </c>
       <c r="BT2" t="inlineStr">
         <is>
-          <t>1 Each</t>
+          <t>Aluminum</t>
         </is>
       </c>
       <c r="BU2" t="inlineStr"/>
       <c r="BV2" t="inlineStr">
         <is>
+          <t>Selling Qty</t>
+        </is>
+      </c>
+      <c r="BW2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BX2" t="inlineStr"/>
+      <c r="BY2" t="inlineStr">
+        <is>
+          <t>Standard Packaging Information</t>
+        </is>
+      </c>
+      <c r="BZ2" t="inlineStr">
+        <is>
+          <t>1 Each</t>
+        </is>
+      </c>
+      <c r="CA2" t="inlineStr"/>
+      <c r="CB2" t="inlineStr">
+        <is>
           <t>Length</t>
         </is>
       </c>
-      <c r="BW2" t="inlineStr">
+      <c r="CC2" t="inlineStr">
         <is>
           <t>2-3/4</t>
         </is>
       </c>
-      <c r="BX2" t="inlineStr">
+      <c r="CD2" t="inlineStr">
         <is>
           <t>in</t>
         </is>
       </c>
-      <c r="BY2" t="inlineStr">
+      <c r="CE2" t="inlineStr">
         <is>
           <t>Width</t>
         </is>
       </c>
-      <c r="BZ2" t="inlineStr">
+      <c r="CF2" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="CA2" t="inlineStr">
+      <c r="CG2" t="inlineStr">
         <is>
           <t>in</t>
         </is>
       </c>
-      <c r="CB2" t="inlineStr">
+      <c r="CH2" t="inlineStr">
         <is>
           <t>Product Type</t>
         </is>
       </c>
-      <c r="CC2" t="inlineStr">
+      <c r="CI2" t="inlineStr">
         <is>
           <t>Sanding Disc</t>
-        </is>
-      </c>
-      <c r="CD2" t="inlineStr"/>
-      <c r="CE2" t="inlineStr">
-        <is>
-          <t>Brand Name</t>
-        </is>
-      </c>
-      <c r="CF2" t="inlineStr">
-        <is>
-          <t>Mirka</t>
-        </is>
-      </c>
-      <c r="CG2" t="inlineStr"/>
-      <c r="CH2" t="inlineStr">
-        <is>
-          <t>Manufacturer Name</t>
-        </is>
-      </c>
-      <c r="CI2" t="inlineStr">
-        <is>
-          <t>Mirka USA Inc</t>
         </is>
       </c>
       <c r="CJ2" t="inlineStr"/>
       <c r="CK2" t="inlineStr">
         <is>
-          <t>Warranty</t>
+          <t>Brand Name</t>
         </is>
       </c>
       <c r="CL2" t="inlineStr">
         <is>
-          <t>1 Year Manufacturer, 1 Year Labor and Parts</t>
+          <t>Mirka</t>
         </is>
       </c>
       <c r="CM2" t="inlineStr"/>
       <c r="CN2" t="inlineStr">
         <is>
-          <t>Standard/Approvals</t>
+          <t>Manufacturer Name</t>
         </is>
       </c>
       <c r="CO2" t="inlineStr">
         <is>
-          <t>ISO 9001 Certified, ANSI Compliant, RoHS Compliant</t>
+          <t>Mirka USA Inc</t>
         </is>
       </c>
       <c r="CP2" t="inlineStr"/>
       <c r="CQ2" t="inlineStr">
         <is>
-          <t>Overall Dimensions</t>
+          <t>Warranty</t>
         </is>
       </c>
       <c r="CR2" t="inlineStr">
         <is>
-          <t>30 in W x 2-3/4 in L</t>
+          <t>1 Year Manufacturer, 1 Year Labor and Parts</t>
         </is>
       </c>
       <c r="CS2" t="inlineStr"/>
       <c r="CT2" t="inlineStr">
         <is>
-          <t>Grit</t>
+          <t>Standard/Approvals</t>
         </is>
       </c>
       <c r="CU2" t="inlineStr">
         <is>
-          <t>P320</t>
+          <t>ISO 9001 Certified, ANSI Compliant, RoHS Compliant</t>
         </is>
       </c>
       <c r="CV2" t="inlineStr"/>
       <c r="CW2" t="inlineStr">
         <is>
-          <t>Grit Standard</t>
+          <t>Overall Dimensions</t>
         </is>
       </c>
       <c r="CX2" t="inlineStr">
         <is>
-          <t>FEPA P-Grade Standard</t>
+          <t>30 in W x 2-3/4 in L</t>
         </is>
       </c>
       <c r="CY2" t="inlineStr"/>
       <c r="CZ2" t="inlineStr">
         <is>
-          <t>Grain Structure</t>
+          <t>Grit Standard</t>
         </is>
       </c>
       <c r="DA2" t="inlineStr">
         <is>
-          <t>Electrostatic Open Mesh Grain Matrix</t>
+          <t>FEPA P-Grade Standard</t>
         </is>
       </c>
       <c r="DB2" t="inlineStr"/>
       <c r="DC2" t="inlineStr">
         <is>
-          <t>Backing Weight</t>
+          <t>Grain Structure</t>
         </is>
       </c>
       <c r="DD2" t="inlineStr">
         <is>
-          <t>Net Mesh (Ultra-Flexible)</t>
+          <t>Electrostatic Open Mesh Grain Matrix</t>
         </is>
       </c>
       <c r="DE2" t="inlineStr"/>
       <c r="DF2" t="inlineStr">
         <is>
-          <t>Bonding Agent</t>
+          <t>Backing Weight</t>
         </is>
       </c>
       <c r="DG2" t="inlineStr">
         <is>
-          <t>Resin Over Resin Bond</t>
+          <t>Net Mesh (Ultra-Flexible)</t>
         </is>
       </c>
       <c r="DH2" t="inlineStr"/>
       <c r="DI2" t="inlineStr">
         <is>
-          <t>Coating Structure</t>
+          <t>Bonding Agent</t>
         </is>
       </c>
       <c r="DJ2" t="inlineStr">
         <is>
-          <t>Net Mesh Permeable Coat</t>
+          <t>Resin Over Resin Bond</t>
         </is>
       </c>
       <c r="DK2" t="inlineStr"/>
       <c r="DL2" t="inlineStr">
         <is>
-          <t>Cutting Action</t>
+          <t>Coating Structure</t>
         </is>
       </c>
       <c r="DM2" t="inlineStr">
         <is>
-          <t>High-Efficiency Dust-Free Smooth Finishing</t>
+          <t>Net Mesh Permeable Coat</t>
         </is>
       </c>
       <c r="DN2" t="inlineStr"/>
       <c r="DO2" t="inlineStr">
         <is>
-          <t>Conformability</t>
+          <t>Cutting Action</t>
         </is>
       </c>
       <c r="DP2" t="inlineStr">
         <is>
-          <t>High Contour Conformability</t>
+          <t>High-Efficiency Dust-Free Smooth Finishing</t>
         </is>
       </c>
       <c r="DQ2" t="inlineStr"/>
       <c r="DR2" t="inlineStr">
         <is>
-          <t>Anti-Clogging Feature</t>
+          <t>Conformability</t>
         </is>
       </c>
       <c r="DS2" t="inlineStr">
         <is>
-          <t>100% Through-Mesh Dust Evacuation</t>
+          <t>High Contour Conformability</t>
         </is>
       </c>
       <c r="DT2" t="inlineStr"/>
       <c r="DU2" t="inlineStr">
         <is>
-          <t>Wet or Dry Application</t>
+          <t>Anti-Clogging Feature</t>
         </is>
       </c>
       <c r="DV2" t="inlineStr">
         <is>
-          <t>Wet and Dry Compatible</t>
+          <t>100% Through-Mesh Dust Evacuation</t>
         </is>
       </c>
       <c r="DW2" t="inlineStr"/>
       <c r="DX2" t="inlineStr">
         <is>
-          <t>Anti-Static Feature</t>
+          <t>Wet or Dry Application</t>
         </is>
       </c>
       <c r="DY2" t="inlineStr">
         <is>
-          <t>Anti-Static Mesh Matrix for Reduced Dust Attraction</t>
+          <t>Wet and Dry Compatible</t>
         </is>
       </c>
       <c r="DZ2" t="inlineStr"/>
       <c r="EA2" t="inlineStr">
         <is>
-          <t>Heat Dissipation</t>
+          <t>Anti-Static Feature</t>
         </is>
       </c>
       <c r="EB2" t="inlineStr">
         <is>
-          <t>Cool Running Formula with Thermal Dissipation</t>
+          <t>Anti-Static Mesh Matrix for Reduced Dust Attraction</t>
         </is>
       </c>
       <c r="EC2" t="inlineStr"/>
       <c r="ED2" t="inlineStr">
         <is>
-          <t>Attachment Type</t>
+          <t>Heat Dissipation</t>
         </is>
       </c>
       <c r="EE2" t="inlineStr">
         <is>
-          <t>Hook and Loop (Grip System)</t>
+          <t>Cool Running Formula with Thermal Dissipation</t>
         </is>
       </c>
       <c r="EF2" t="inlineStr"/>
       <c r="EG2" t="inlineStr">
         <is>
-          <t>Hole Pattern</t>
+          <t>Attachment Type</t>
         </is>
       </c>
       <c r="EH2" t="inlineStr">
         <is>
-          <t>Dust-Free Net Mesh Permeable Surface</t>
+          <t>Hook and Loop (Grip System)</t>
         </is>
       </c>
       <c r="EI2" t="inlineStr"/>
       <c r="EJ2" t="inlineStr">
         <is>
-          <t>Compatible Tools</t>
+          <t>Hole Pattern</t>
         </is>
       </c>
       <c r="EK2" t="inlineStr">
         <is>
-          <t>Random Orbital Sander, Hand Sanding Block, File Sander</t>
+          <t>Dust-Free Net Mesh Permeable Surface</t>
         </is>
       </c>
       <c r="EL2" t="inlineStr"/>
       <c r="EM2" t="inlineStr">
         <is>
-          <t>Mounting Configuration</t>
+          <t>Compatible Tools</t>
         </is>
       </c>
       <c r="EN2" t="inlineStr">
         <is>
-          <t>Quick-Change Grip Pad Mounting</t>
+          <t>Random Orbital Sander, Hand Sanding Block, File Sander</t>
         </is>
       </c>
       <c r="EO2" t="inlineStr"/>
       <c r="EP2" t="inlineStr">
         <is>
-          <t>Primary Workpiece Substrate</t>
+          <t>Mounting Configuration</t>
         </is>
       </c>
       <c r="EQ2" t="inlineStr">
         <is>
-          <t>Hardwood, Softwood, Primers &amp; Automotive Paint</t>
+          <t>Quick-Change Grip Pad Mounting</t>
         </is>
       </c>
       <c r="ER2" t="inlineStr"/>
       <c r="ES2" t="inlineStr">
         <is>
-          <t>Secondary Workpiece Substrate</t>
+          <t>Primary Workpiece Substrate</t>
         </is>
       </c>
       <c r="ET2" t="inlineStr">
         <is>
-          <t>Solid Surface Polymers, Gel Coats, Composites</t>
+          <t>Hardwood, Softwood, Primers &amp; Automotive Paint</t>
         </is>
       </c>
       <c r="EU2" t="inlineStr"/>
       <c r="EV2" t="inlineStr">
         <is>
-          <t>Target Surface Finish</t>
+          <t>Secondary Workpiece Substrate</t>
         </is>
       </c>
       <c r="EW2" t="inlineStr">
         <is>
-          <t>Ultra-Fine Scratch-Free Finish</t>
+          <t>Solid Surface Polymers, Gel Coats, Composites</t>
         </is>
       </c>
       <c r="EX2" t="inlineStr"/>
       <c r="EY2" t="inlineStr">
         <is>
-          <t>Primary Function</t>
+          <t>Target Surface Finish</t>
         </is>
       </c>
       <c r="EZ2" t="inlineStr">
         <is>
-          <t>Dust-Free Fine Finish Sanding</t>
+          <t>Ultra-Fine Scratch-Free Finish</t>
         </is>
       </c>
       <c r="FA2" t="inlineStr"/>
       <c r="FB2" t="inlineStr">
         <is>
-          <t>Package Quantity</t>
+          <t>Primary Function</t>
         </is>
       </c>
       <c r="FC2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Dust-Free Fine Finish Sanding</t>
         </is>
       </c>
       <c r="FD2" t="inlineStr"/>
       <c r="FE2" t="inlineStr">
         <is>
-          <t>Package Type</t>
+          <t>Package Quantity</t>
         </is>
       </c>
       <c r="FF2" t="inlineStr">
         <is>
-          <t>Grip Roll in Dispenser Carton</t>
+          <t>1</t>
         </is>
       </c>
       <c r="FG2" t="inlineStr"/>
       <c r="FH2" t="inlineStr">
         <is>
+          <t>Package Type</t>
+        </is>
+      </c>
+      <c r="FI2" t="inlineStr">
+        <is>
+          <t>Grip Roll in Dispenser Carton</t>
+        </is>
+      </c>
+      <c r="FJ2" t="inlineStr"/>
+      <c r="FK2" t="inlineStr">
+        <is>
           <t>Unit Packaging Weight</t>
         </is>
       </c>
-      <c r="FI2" t="inlineStr">
+      <c r="FL2" t="inlineStr">
         <is>
           <t>1.2</t>
         </is>
       </c>
-      <c r="FJ2" t="inlineStr">
+      <c r="FM2" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
       </c>
-      <c r="FK2" t="inlineStr">
+      <c r="FN2" t="inlineStr">
         <is>
           <t>Country Of Origin</t>
         </is>
       </c>
-      <c r="FL2" t="inlineStr">
+      <c r="FO2" t="inlineStr">
         <is>
           <t>Finland</t>
-        </is>
-      </c>
-      <c r="FM2" t="inlineStr"/>
-      <c r="FN2" t="inlineStr">
-        <is>
-          <t>Discontinued</t>
-        </is>
-      </c>
-      <c r="FO2" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
       <c r="FP2" t="inlineStr"/>
       <c r="FQ2" t="inlineStr">
         <is>
-          <t>Safety Standard</t>
+          <t>Discontinued</t>
         </is>
       </c>
       <c r="FR2" t="inlineStr">
         <is>
-          <t>OSHA Safety Standard Compliant</t>
+          <t>No</t>
         </is>
       </c>
       <c r="FS2" t="inlineStr"/>
       <c r="FT2" t="inlineStr">
         <is>
-          <t>Quality Certification</t>
+          <t>Safety Standard</t>
         </is>
       </c>
       <c r="FU2" t="inlineStr">
         <is>
-          <t>ISO 9001:2015 Quality Management System</t>
+          <t>OSHA Safety Standard Compliant</t>
         </is>
       </c>
       <c r="FV2" t="inlineStr"/>
       <c r="FW2" t="inlineStr">
         <is>
-          <t>Environmental Compliance</t>
+          <t>Quality Certification</t>
         </is>
       </c>
       <c r="FX2" t="inlineStr">
         <is>
-          <t>RoHS Directive 2011/65/EU Compliant</t>
+          <t>ISO 9001:2015 Quality Management System</t>
         </is>
       </c>
       <c r="FY2" t="inlineStr"/>
       <c r="FZ2" t="inlineStr">
         <is>
-          <t>Prop 65</t>
+          <t>Environmental Compliance</t>
         </is>
       </c>
       <c r="GA2" t="inlineStr">
         <is>
-          <t>WARNING: Cancer and Reproductive Harm - www.P65Warnings.ca.gov</t>
+          <t>RoHS Directive 2011/65/EU Compliant</t>
         </is>
       </c>
       <c r="GB2" t="inlineStr"/>
       <c r="GC2" t="inlineStr">
         <is>
-          <t>Manufacturer Part Number</t>
+          <t>Prop 65</t>
         </is>
       </c>
       <c r="GD2" t="inlineStr">
         <is>
-          <t>9A-570-320</t>
+          <t>WARNING: Cancer and Reproductive Harm - www.P65Warnings.ca.gov</t>
         </is>
       </c>
       <c r="GE2" t="inlineStr"/>
       <c r="GF2" t="inlineStr">
         <is>
-          <t>Color</t>
+          <t>Manufacturer Part Number</t>
         </is>
       </c>
       <c r="GG2" t="inlineStr">
         <is>
-          <t>Grey / Mesh Brown</t>
+          <t>9A-570-320</t>
         </is>
       </c>
       <c r="GH2" t="inlineStr"/>
       <c r="GI2" t="inlineStr">
         <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="GJ2" t="inlineStr">
+        <is>
+          <t>Grey / Mesh Brown</t>
+        </is>
+      </c>
+      <c r="GK2" t="inlineStr"/>
+      <c r="GL2" t="inlineStr">
+        <is>
           <t>Selling UOM</t>
         </is>
       </c>
-      <c r="GJ2" t="inlineStr">
+      <c r="GM2" t="inlineStr">
         <is>
           <t>Each</t>
         </is>
       </c>
-      <c r="GK2" t="inlineStr"/>
-      <c r="GL2" t="inlineStr"/>
-      <c r="GM2" t="inlineStr"/>
       <c r="GN2" t="inlineStr"/>
       <c r="GO2" t="inlineStr"/>
       <c r="GP2" t="inlineStr"/>
@@ -2683,22 +2691,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://www.toolmarts.com/freud-dbd090094101f-diablo-9-in-metal-cut-off-disc</t>
+          <t>https://www.qualityworldtools.com/product/freud-dbd090094101f-diablo-9-in-metal-cut-off-disc/</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.toolmarts.com/freud-dbd090094101f-diablo-9-in-metal-cut-off-disc</t>
+          <t>https://www.qualityworldtools.com/product/freud-dbd090094101f-diablo-9-in-metal-cut-off-disc/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://shopkoopman.com/collections/freud-america-inc?page=2</t>
+          <t>https://www.freudsharpening.com/product/diablo-9-in-metal-cut-off-disc/316070</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.toolmarts.com/freud-dbd090094101f-diablo-9-in-metal-cut-off-disc/documents/DBD090094101F_manual.pdf</t>
+          <t>https://www.qualityworldtools.com/product/freud-dbd090094101f-diablo-9-in-metal-cut-off-disc//documents/DBD090094101F_manual.pdf</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -3087,7 +3095,7 @@
       </c>
       <c r="CO3" t="inlineStr">
         <is>
-          <t>19/32</t>
+          <t>9</t>
         </is>
       </c>
       <c r="CP3" t="inlineStr">
@@ -3132,7 +3140,7 @@
       </c>
       <c r="CX3" t="inlineStr">
         <is>
-          <t>19/32 in Dia x .045 in T</t>
+          <t>9 in Dia x .045 in T</t>
         </is>
       </c>
       <c r="CY3" t="inlineStr"/>

</xml_diff>